<commit_message>
sqlite with pandas dataframe.
</commit_message>
<xml_diff>
--- a/python/output/network_report.xlsx
+++ b/python/output/network_report.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ip_interface_bri" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ip_ospf_neighbor" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -717,203 +716,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>hostname</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>neighbor_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>dead_time</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ip_address</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>interface</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Router-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>10.0.0.3</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FULL/DROTHER</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>00:00:31</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>10.0.0.3</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Ethernet0/1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Router-01</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>10.255.0.2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FULL/DR</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>00:00:33</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>10.0.0.2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Ethernet0/1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Router-02</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>10.0.0.3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>FULL/DROTHER</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>00:00:38</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>10.0.0.3</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Ethernet0/1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Router-02</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>10.255.0.1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>FULL/BDR</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>00:00:32</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>10.0.0.1</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Ethernet0/1</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>